<commit_message>
Fix 2026 validation PDF portability on Windows
</commit_message>
<xml_diff>
--- a/validation_2026_age32/edge_validation.xlsx
+++ b/validation_2026_age32/edge_validation.xlsx
@@ -3842,7 +3842,7 @@
       </c>
       <c r="C2" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0001691826002933-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0001691826002933-main.pdf</t>
         </is>
       </c>
       <c r="D2" t="inlineStr" s="0">
@@ -3879,7 +3879,7 @@
       </c>
       <c r="C3" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0001691826006839-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0001691826006839-main.pdf</t>
         </is>
       </c>
       <c r="D3" t="inlineStr" s="0">
@@ -3916,7 +3916,7 @@
       </c>
       <c r="C4" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0001691826009352-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0001691826009352-main.pdf</t>
         </is>
       </c>
       <c r="D4" t="inlineStr" s="0">
@@ -3953,7 +3953,7 @@
       </c>
       <c r="C5" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0005796726000781-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0005796726000781-main.pdf</t>
         </is>
       </c>
       <c r="D5" t="inlineStr" s="0">
@@ -3990,7 +3990,7 @@
       </c>
       <c r="C6" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0006322325015306-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0006322325015306-main.pdf</t>
         </is>
       </c>
       <c r="D6" t="inlineStr" s="0">
@@ -4027,7 +4027,7 @@
       </c>
       <c r="C7" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0022395625006776.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0022395625006776.pdf</t>
         </is>
       </c>
       <c r="D7" t="inlineStr" s="0">
@@ -4064,7 +4064,7 @@
       </c>
       <c r="C8" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0022395625007563.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0022395625007563.pdf</t>
         </is>
       </c>
       <c r="D8" t="inlineStr" s="0">
@@ -4101,7 +4101,7 @@
       </c>
       <c r="C9" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0022395626000300.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0022395626000300.pdf</t>
         </is>
       </c>
       <c r="D9" t="inlineStr" s="0">
@@ -4138,7 +4138,7 @@
       </c>
       <c r="C10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0022395626000506.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0022395626000506.pdf</t>
         </is>
       </c>
       <c r="D10" t="inlineStr" s="0">
@@ -4175,7 +4175,7 @@
       </c>
       <c r="C11" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0033350626001411.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0033350626001411.pdf</t>
         </is>
       </c>
       <c r="D11" t="inlineStr" s="0">
@@ -4212,7 +4212,7 @@
       </c>
       <c r="C12" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0147651326004987-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0147651326004987-main.pdf</t>
         </is>
       </c>
       <c r="D12" t="inlineStr" s="0">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="C13" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0149763426000254-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0149763426000254-main.pdf</t>
         </is>
       </c>
       <c r="D13" t="inlineStr" s="0">
@@ -4286,7 +4286,7 @@
       </c>
       <c r="C14" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0149763426001806-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0149763426001806-main.pdf</t>
         </is>
       </c>
       <c r="D14" t="inlineStr" s="0">
@@ -4323,7 +4323,7 @@
       </c>
       <c r="C15" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0163834326000253.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0163834326000253.pdf</t>
         </is>
       </c>
       <c r="D15" t="inlineStr" s="0">
@@ -4360,7 +4360,7 @@
       </c>
       <c r="C16" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165032725016106-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165032725016106-main.pdf</t>
         </is>
       </c>
       <c r="D16" t="inlineStr" s="0">
@@ -4397,7 +4397,7 @@
       </c>
       <c r="C17" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165032725017641-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165032725017641-main.pdf</t>
         </is>
       </c>
       <c r="D17" t="inlineStr" s="0">
@@ -4434,7 +4434,7 @@
       </c>
       <c r="C18" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S016503272502172X-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S016503272502172X-main.pdf</t>
         </is>
       </c>
       <c r="D18" t="inlineStr" s="0">
@@ -4471,7 +4471,7 @@
       </c>
       <c r="C19" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165032725025492-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165032725025492-main.pdf</t>
         </is>
       </c>
       <c r="D19" t="inlineStr" s="0">
@@ -4508,7 +4508,7 @@
       </c>
       <c r="C20" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165032726000984-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165032726000984-main.pdf</t>
         </is>
       </c>
       <c r="D20" t="inlineStr" s="0">
@@ -4545,7 +4545,7 @@
       </c>
       <c r="C21" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165032726009894-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165032726009894-main.pdf</t>
         </is>
       </c>
       <c r="D21" t="inlineStr" s="0">
@@ -4582,7 +4582,7 @@
       </c>
       <c r="C22" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165178125005293-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165178125005293-main.pdf</t>
         </is>
       </c>
       <c r="D22" t="inlineStr" s="0">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="C23" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165178126000363-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165178126000363-main.pdf</t>
         </is>
       </c>
       <c r="D23" t="inlineStr" s="0">
@@ -4656,7 +4656,7 @@
       </c>
       <c r="C24" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165178126001460-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165178126001460-main.pdf</t>
         </is>
       </c>
       <c r="D24" t="inlineStr" s="0">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="C25" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0165178126003276-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0165178126003276-main.pdf</t>
         </is>
       </c>
       <c r="D25" t="inlineStr" s="0">
@@ -4730,7 +4730,7 @@
       </c>
       <c r="C26" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0272735825001552-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0272735825001552-main.pdf</t>
         </is>
       </c>
       <c r="D26" t="inlineStr" s="0">
@@ -4767,7 +4767,7 @@
       </c>
       <c r="C27" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0277953626006258-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0277953626006258-main.pdf</t>
         </is>
       </c>
       <c r="D27" t="inlineStr" s="0">
@@ -4804,7 +4804,7 @@
       </c>
       <c r="C28" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0387760426000343.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0387760426000343.pdf</t>
         </is>
       </c>
       <c r="D28" t="inlineStr" s="0">
@@ -4841,7 +4841,7 @@
       </c>
       <c r="C29" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S088259632600151X-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S088259632600151X-main.pdf</t>
         </is>
       </c>
       <c r="D29" t="inlineStr" s="0">
@@ -4878,7 +4878,7 @@
       </c>
       <c r="C30" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0890856725002151-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0890856725002151-main.pdf</t>
         </is>
       </c>
       <c r="D30" t="inlineStr" s="0">
@@ -4915,7 +4915,7 @@
       </c>
       <c r="C31" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0890856725003399-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0890856725003399-main.pdf</t>
         </is>
       </c>
       <c r="D31" t="inlineStr" s="0">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="C32" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0890856725020519-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0890856725020519-main.pdf</t>
         </is>
       </c>
       <c r="D32" t="inlineStr" s="0">
@@ -4989,7 +4989,7 @@
       </c>
       <c r="C33" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0891422226000715-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0891422226000715-main.pdf</t>
         </is>
       </c>
       <c r="D33" t="inlineStr" s="0">
@@ -5026,7 +5026,7 @@
       </c>
       <c r="C34" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S089142222600137X-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S089142222600137X-main.pdf</t>
         </is>
       </c>
       <c r="D34" t="inlineStr" s="0">
@@ -5063,7 +5063,7 @@
       </c>
       <c r="C35" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0925492726001502.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0925492726001502.pdf</t>
         </is>
       </c>
       <c r="D35" t="inlineStr" s="0">
@@ -5100,7 +5100,7 @@
       </c>
       <c r="C36" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S0929693X26001296-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S0929693X26001296-main.pdf</t>
         </is>
       </c>
       <c r="D36" t="inlineStr" s="0">
@@ -5137,7 +5137,7 @@
       </c>
       <c r="C37" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S1087079226000754-main (1).pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S1087079226000754-main (1).pdf</t>
         </is>
       </c>
       <c r="D37" t="inlineStr" s="0">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="C38" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S1087079226000754-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S1087079226000754-main.pdf</t>
         </is>
       </c>
       <c r="D38" t="inlineStr" s="0">
@@ -5211,7 +5211,7 @@
       </c>
       <c r="C39" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S1386505626001577.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S1386505626001577.pdf</t>
         </is>
       </c>
       <c r="D39" t="inlineStr" s="0">
@@ -5248,7 +5248,7 @@
       </c>
       <c r="C40" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S1389945726003771-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S1389945726003771-main.pdf</t>
         </is>
       </c>
       <c r="D40" t="inlineStr" s="0">
@@ -5285,7 +5285,7 @@
       </c>
       <c r="C41" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S152550502500592X.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S152550502500592X.pdf</t>
         </is>
       </c>
       <c r="D41" t="inlineStr" s="0">
@@ -5322,7 +5322,7 @@
       </c>
       <c r="C42" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S1525505026000867.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S1525505026000867.pdf</t>
         </is>
       </c>
       <c r="D42" t="inlineStr" s="0">
@@ -5359,7 +5359,7 @@
       </c>
       <c r="C43" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S1878929326000575-main.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S1878929326000575-main.pdf</t>
         </is>
       </c>
       <c r="D43" t="inlineStr" s="0">
@@ -5396,7 +5396,7 @@
       </c>
       <c r="C44" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/1-s2.0-S221503662600091X.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/1-s2.0-S221503662600091X.pdf</t>
         </is>
       </c>
       <c r="D44" t="inlineStr" s="0">
@@ -5433,7 +5433,7 @@
       </c>
       <c r="C45" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/167.full.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/167.full.pdf</t>
         </is>
       </c>
       <c r="D45" t="inlineStr" s="0">
@@ -5470,7 +5470,7 @@
       </c>
       <c r="C46" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/31_26-00080.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/31_26-00080.pdf</t>
         </is>
       </c>
       <c r="D46" t="inlineStr" s="0">
@@ -5507,7 +5507,7 @@
       </c>
       <c r="C47" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/784.full.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/784.full.pdf</t>
         </is>
       </c>
       <c r="D47" t="inlineStr" s="0">
@@ -5544,7 +5544,7 @@
       </c>
       <c r="C48" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/A Meta-Analysis of the Prevalence of ADHD in Youth Across Racial and Ethnic Groups.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/A Meta-Analysis of the Prevalence of ADHD in Youth Across Racial and Ethnic Groups.pdf</t>
         </is>
       </c>
       <c r="D48" t="inlineStr" s="0">
@@ -5581,7 +5581,7 @@
       </c>
       <c r="C49" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/A multi stakeholder preliminary needs assessment to inform the co design of a digital telerehabilitation tool for children and adolescents with ADHD.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/A multi stakeholder preliminary needs assessment to inform the co design of a digital telerehabilitation tool for children and adolescents with ADHD.pdf</t>
         </is>
       </c>
       <c r="D49" t="inlineStr" s="0">
@@ -5618,7 +5618,7 @@
       </c>
       <c r="C50" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Basic Clin Pharma Tox - 2026 - Sonne - Regional Variation in ADHD Treatment and Diagnosis Among Children and Adolescents in.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Basic Clin Pharma Tox - 2026 - Sonne - Regional Variation in ADHD Treatment and Diagnosis Among Children and Adolescents in.pdf</t>
         </is>
       </c>
       <c r="D50" t="inlineStr" s="0">
@@ -5655,7 +5655,7 @@
       </c>
       <c r="C51" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Child - 2025 - Denis - Parenting Practices in Families of Children With Comorbid ADHD and Anxiety Disorders  A Systematic.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Child - 2025 - Denis - Parenting Practices in Families of Children With Comorbid ADHD and Anxiety Disorders  A Systematic.pdf</t>
         </is>
       </c>
       <c r="D51" t="inlineStr" s="0">
@@ -5692,7 +5692,7 @@
       </c>
       <c r="C52" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Child - 2025 - Tang - Barriers to and Enablers of the Transition From Child to Adult Mental Health Services for Autistic.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Child - 2025 - Tang - Barriers to and Enablers of the Transition From Child to Adult Mental Health Services for Autistic.pdf</t>
         </is>
       </c>
       <c r="D52" t="inlineStr" s="0">
@@ -5729,7 +5729,7 @@
       </c>
       <c r="C53" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Child - 2026 - Smith - Mind the Gap  Sleep Problems in Children With ADHD A Qualitative Analysis of Clinician Training.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Child - 2026 - Smith - Mind the Gap  Sleep Problems in Children With ADHD A Qualitative Analysis of Clinician Training.pdf</t>
         </is>
       </c>
       <c r="D53" t="inlineStr" s="0">
@@ -5766,7 +5766,7 @@
       </c>
       <c r="C54" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Child Psychology Psychiatry - 2025 - Shakeshaft - Mapping phenotypic and genetic relationships among irritability .pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Child Psychology Psychiatry - 2025 - Shakeshaft - Mapping phenotypic and genetic relationships among irritability .pdf</t>
         </is>
       </c>
       <c r="D54" t="inlineStr" s="0">
@@ -5803,7 +5803,7 @@
       </c>
       <c r="C55" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Child Psychology Psychiatry - 2025 - You - The role of comorbid childhood mental health and neurodevelopmental conditions.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Child Psychology Psychiatry - 2025 - You - The role of comorbid childhood mental health and neurodevelopmental conditions.pdf</t>
         </is>
       </c>
       <c r="D55" t="inlineStr" s="0">
@@ -5840,7 +5840,7 @@
       </c>
       <c r="C56" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Child Psychology Psychiatry - 2026 - Thomson - Editorial  ADHD persistence   the interplay of genes  socioeconomic context .pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Child Psychology Psychiatry - 2026 - Thomson - Editorial  ADHD persistence   the interplay of genes  socioeconomic context .pdf</t>
         </is>
       </c>
       <c r="D56" t="inlineStr" s="0">
@@ -5877,7 +5877,7 @@
       </c>
       <c r="C57" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Do Children and Adolescents with Attention Deficit Hyperactivity Disorder Use Screens More  A Systematic Review and Meta-Analysis.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Do Children and Adolescents with Attention Deficit Hyperactivity Disorder Use Screens More  A Systematic Review and Meta-Analysis.pdf</t>
         </is>
       </c>
       <c r="D57" t="inlineStr" s="0">
@@ -5914,7 +5914,7 @@
       </c>
       <c r="C58" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Do Wechsler intelligence scales predict academic achievement in children with ADHD or autism  A systematic review and meta-analysis.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Do Wechsler intelligence scales predict academic achievement in children with ADHD or autism  A systematic review and meta-analysis.pdf</t>
         </is>
       </c>
       <c r="D58" t="inlineStr" s="0">
@@ -5951,7 +5951,7 @@
       </c>
       <c r="C59" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Early Intervention Psych - 2026 - Ricci - Neurodevelopmental  Pharmacological and Substance Use Factors in the Association.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Early Intervention Psych - 2026 - Ricci - Neurodevelopmental  Pharmacological and Substance Use Factors in the Association.pdf</t>
         </is>
       </c>
       <c r="D59" t="inlineStr" s="0">
@@ -5988,7 +5988,7 @@
       </c>
       <c r="C60" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Family Process - 2026 - Guerin - The Stigmatization of Caregivers of Children With Attention‐Deficit Hyperactivity Disorder.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Family Process - 2026 - Guerin - The Stigmatization of Caregivers of Children With Attention‐Deficit Hyperactivity Disorder.pdf</t>
         </is>
       </c>
       <c r="D60" t="inlineStr" s="0">
@@ -6025,7 +6025,7 @@
       </c>
       <c r="C61" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Int J Methods Psych Res - 2026 - Assaf - Psychometric Assessment of the Arabic Translation of the Adult ADHD Self‐Report.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Int J Methods Psych Res - 2026 - Assaf - Psychometric Assessment of the Arabic Translation of the Adult ADHD Self‐Report.pdf</t>
         </is>
       </c>
       <c r="D61" t="inlineStr" s="0">
@@ -6062,7 +6062,7 @@
       </c>
       <c r="C62" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/J Human Nutrition Diet - 2026 - Sadowska - Gut Microbiome and ADHD  A Narrative Review of Clinical Evidence and Practice.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/J Human Nutrition Diet - 2026 - Sadowska - Gut Microbiome and ADHD  A Narrative Review of Clinical Evidence and Practice.pdf</t>
         </is>
       </c>
       <c r="D62" t="inlineStr" s="0">
@@ -6099,7 +6099,7 @@
       </c>
       <c r="C63" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/J Marital Family Therapy - 2025 - O'Brien - I Felt Like a Burden   An Exploration Into the Experience of Romantic.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/J Marital Family Therapy - 2025 - O'Brien - I Felt Like a Burden   An Exploration Into the Experience of Romantic.pdf</t>
         </is>
       </c>
       <c r="D63" t="inlineStr" s="0">
@@ -6136,7 +6136,7 @@
       </c>
       <c r="C64" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/J Paediatrics Child Health - 2026 - Pehlevan - Parental Knowledge and Recognition of Preschool Manifestations of ADHD in.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/J Paediatrics Child Health - 2026 - Pehlevan - Parental Knowledge and Recognition of Preschool Manifestations of ADHD in.pdf</t>
         </is>
       </c>
       <c r="D64" t="inlineStr" s="0">
@@ -6173,7 +6173,7 @@
       </c>
       <c r="C65" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Medical Journal of Australia - 2026 - Morgan - Stigmatising Attitudes Towards People With Depression  Bipolar Disorder .pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Medical Journal of Australia - 2026 - Morgan - Stigmatising Attitudes Towards People With Depression  Bipolar Disorder .pdf</t>
         </is>
       </c>
       <c r="D65" t="inlineStr" s="0">
@@ -6210,7 +6210,7 @@
       </c>
       <c r="C66" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Medical Journal of Australia - 2026 - Ouliaris - ADHD Across the Lifespan  Reconsidering Assumptions of Diagnostic.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Medical Journal of Australia - 2026 - Ouliaris - ADHD Across the Lifespan  Reconsidering Assumptions of Diagnostic.pdf</t>
         </is>
       </c>
       <c r="D66" t="inlineStr" s="0">
@@ -6247,7 +6247,7 @@
       </c>
       <c r="C67" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Prevalence of the Prescribing of Attention-Deficit Hyperactivity Disorder Medication During Pregnancy  A Systematic Review.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Prevalence of the Prescribing of Attention-Deficit Hyperactivity Disorder Medication During Pregnancy  A Systematic Review.pdf</t>
         </is>
       </c>
       <c r="D67" t="inlineStr" s="0">
@@ -6284,7 +6284,7 @@
       </c>
       <c r="C68" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/SHTI-336-SHTI260681.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/SHTI-336-SHTI260681.pdf</t>
         </is>
       </c>
       <c r="D68" t="inlineStr" s="0">
@@ -6321,7 +6321,7 @@
       </c>
       <c r="C69" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Scandinavian J Psychology - 2025 - Isaksson - Feasibility of the Psychoeducational Programme SKILLS for the Child s Social.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Scandinavian J Psychology - 2025 - Isaksson - Feasibility of the Psychoeducational Programme SKILLS for the Child s Social.pdf</t>
         </is>
       </c>
       <c r="D69" t="inlineStr" s="0">
@@ -6358,7 +6358,7 @@
       </c>
       <c r="C70" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/Scandinavian Med Sci Sports - 2026 - Liang - The Effects of Physical Activity Timing and Adherence to Physical Activity.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/Scandinavian Med Sci Sports - 2026 - Liang - The Effects of Physical Activity Timing and Adherence to Physical Activity.pdf</t>
         </is>
       </c>
       <c r="D70" t="inlineStr" s="0">
@@ -6395,7 +6395,7 @@
       </c>
       <c r="C71" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/a-2689-4911.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/a-2689-4911.pdf</t>
         </is>
       </c>
       <c r="D71" t="inlineStr" s="0">
@@ -6432,7 +6432,7 @@
       </c>
       <c r="C72" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/acag057.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/acag057.pdf</t>
         </is>
       </c>
       <c r="D72" t="inlineStr" s="0">
@@ -6469,7 +6469,7 @@
       </c>
       <c r="C73" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/acs.est.6c01402.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/acs.est.6c01402.pdf</t>
         </is>
       </c>
       <c r="D73" t="inlineStr" s="0">
@@ -6506,7 +6506,7 @@
       </c>
       <c r="C74" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/altunkılıc-et-al-2026-the-effect-of-methylphenidate-treatment-on-oxidative-stress-levels-in-children-diagnosed-with.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/altunkılıc-et-al-2026-the-effect-of-methylphenidate-treatment-on-oxidative-stress-levels-in-children-diagnosed-with.pdf</t>
         </is>
       </c>
       <c r="D74" t="inlineStr" s="0">
@@ -6543,7 +6543,7 @@
       </c>
       <c r="C75" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/bsr-2025-4061.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/bsr-2025-4061.pdf</t>
         </is>
       </c>
       <c r="D75" t="inlineStr" s="0">
@@ -6580,7 +6580,7 @@
       </c>
       <c r="C76" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/bussanich-et-al-2025-school-based-social-skills-interventions-for-youth-with-adhd-a-systematic-review-and-meta-analysis.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/bussanich-et-al-2025-school-based-social-skills-interventions-for-youth-with-adhd-a-systematic-review-and-meta-analysis.pdf</t>
         </is>
       </c>
       <c r="D76" t="inlineStr" s="0">
@@ -6617,7 +6617,7 @@
       </c>
       <c r="C77" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/download.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/download.pdf</t>
         </is>
       </c>
       <c r="D77" t="inlineStr" s="0">
@@ -6654,7 +6654,7 @@
       </c>
       <c r="C78" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/e119568.full.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/e119568.full.pdf</t>
         </is>
       </c>
       <c r="D78" t="inlineStr" s="0">
@@ -6691,7 +6691,7 @@
       </c>
       <c r="C79" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/formative-2026-1-e82164.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/formative-2026-1-e82164.pdf</t>
         </is>
       </c>
       <c r="D79" t="inlineStr" s="0">
@@ -6728,7 +6728,7 @@
       </c>
       <c r="C80" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/hill-et-al-2025-narrative-and-non-narrative-discourse-skills-in-adhd-across-the-lifespan-a-systematic-review-of-the.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/hill-et-al-2025-narrative-and-non-narrative-discourse-skills-in-adhd-across-the-lifespan-a-systematic-review-of-the.pdf</t>
         </is>
       </c>
       <c r="D80" t="inlineStr" s="0">
@@ -6765,7 +6765,7 @@
       </c>
       <c r="C81" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/hoskins-et-al-2026-symptoms-of-anxiety-in-adults-with-adhd-a-systematic-review-and-meta-analysis-of-case-control-studies.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/hoskins-et-al-2026-symptoms-of-anxiety-in-adults-with-adhd-a-systematic-review-and-meta-analysis-of-case-control-studies.pdf</t>
         </is>
       </c>
       <c r="D81" t="inlineStr" s="0">
@@ -6802,7 +6802,7 @@
       </c>
       <c r="C82" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/ijms-27-03453-v3.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/ijms-27-03453-v3.pdf</t>
         </is>
       </c>
       <c r="D82" t="inlineStr" s="0">
@@ -6839,7 +6839,7 @@
       </c>
       <c r="C83" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/jamainternal_luo_2026_oi_260035_1788184625.4213.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/jamainternal_luo_2026_oi_260035_1788184625.4213.pdf</t>
         </is>
       </c>
       <c r="D83" t="inlineStr" s="0">
@@ -6876,7 +6876,7 @@
       </c>
       <c r="C84" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/jamapsychiatry_labianca_2026_oi_260031_1788289932.03306.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/jamapsychiatry_labianca_2026_oi_260031_1788289932.03306.pdf</t>
         </is>
       </c>
       <c r="D84" t="inlineStr" s="0">
@@ -6913,7 +6913,7 @@
       </c>
       <c r="C85" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/jamapsychiatry_pan_2026_oi_260001_1777052922.67615.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/jamapsychiatry_pan_2026_oi_260001_1777052922.67615.pdf</t>
         </is>
       </c>
       <c r="D85" t="inlineStr" s="0">
@@ -6950,7 +6950,7 @@
       </c>
       <c r="C86" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/jamapsychiatry_volotinen_2026_oi_260011_1779900161.36996.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/jamapsychiatry_volotinen_2026_oi_260011_1779900161.36996.pdf</t>
         </is>
       </c>
       <c r="D86" t="inlineStr" s="0">
@@ -6987,7 +6987,7 @@
       </c>
       <c r="C87" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/jmir-2026-1-e95043.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/jmir-2026-1-e95043.pdf</t>
         </is>
       </c>
       <c r="D87" t="inlineStr" s="0">
@@ -7024,7 +7024,7 @@
       </c>
       <c r="C88" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/jogh-16-04233n.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/jogh-16-04233n.pdf</t>
         </is>
       </c>
       <c r="D88" t="inlineStr" s="0">
@@ -7061,7 +7061,7 @@
       </c>
       <c r="C89" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/journal.pone.0314669.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/journal.pone.0314669.pdf</t>
         </is>
       </c>
       <c r="D89" t="inlineStr" s="0">
@@ -7098,7 +7098,7 @@
       </c>
       <c r="C90" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/journal.pone.0341817.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/journal.pone.0341817.pdf</t>
         </is>
       </c>
       <c r="D90" t="inlineStr" s="0">
@@ -7135,7 +7135,7 @@
       </c>
       <c r="C91" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/journal.pone.0356825.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/journal.pone.0356825.pdf</t>
         </is>
       </c>
       <c r="D91" t="inlineStr" s="0">
@@ -7172,7 +7172,7 @@
       </c>
       <c r="C92" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/journal.pone.0357837.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/journal.pone.0357837.pdf</t>
         </is>
       </c>
       <c r="D92" t="inlineStr" s="0">
@@ -7209,7 +7209,7 @@
       </c>
       <c r="C93" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/karimi-et-al-2025-treatment-adherence-in-adhd-a-systematic-review-of-influencing-factors-and-strategies-for-improvement.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/karimi-et-al-2025-treatment-adherence-in-adhd-a-systematic-review-of-influencing-factors-and-strategies-for-improvement.pdf</t>
         </is>
       </c>
       <c r="D93" t="inlineStr" s="0">
@@ -7246,7 +7246,7 @@
       </c>
       <c r="C94" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/leffa_2026_oi_260927_1788960869.95197.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/leffa_2026_oi_260927_1788960869.95197.pdf</t>
         </is>
       </c>
       <c r="D94" t="inlineStr" s="0">
@@ -7283,7 +7283,7 @@
       </c>
       <c r="C95" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/leow-et-al-2026-association-between-attention-deficit-hyperactivity-disorder-and-obstructive-sleep-apnea-in-children-a.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/leow-et-al-2026-association-between-attention-deficit-hyperactivity-disorder-and-obstructive-sleep-apnea-in-children-a.pdf</t>
         </is>
       </c>
       <c r="D95" t="inlineStr" s="0">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="C96" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/liang-et-al-2025-the-family-quality-of-life-of-children-with-specific-learning-disabilities-attention-deficit.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/liang-et-al-2025-the-family-quality-of-life-of-children-with-specific-learning-disabilities-attention-deficit.pdf</t>
         </is>
       </c>
       <c r="D96" t="inlineStr" s="0">
@@ -7357,7 +7357,7 @@
       </c>
       <c r="C97" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/longitudinal-associations-among-autism-and-adhd-traits-social-maladjustment-and-mental-health-in-school-aged-children.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/longitudinal-associations-among-autism-and-adhd-traits-social-maladjustment-and-mental-health-in-school-aged-children.pdf</t>
         </is>
       </c>
       <c r="D97" t="inlineStr" s="0">
@@ -7394,7 +7394,7 @@
       </c>
       <c r="C98" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/madsen-et-al-2025-maternal-adhd-diagnoses-before-and-after-childbirth-a-danish-population-based-cohort-study.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/madsen-et-al-2025-maternal-adhd-diagnoses-before-and-after-childbirth-a-danish-population-based-cohort-study.pdf</t>
         </is>
       </c>
       <c r="D98" t="inlineStr" s="0">
@@ -7431,7 +7431,7 @@
       </c>
       <c r="C99" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/mctaggart-et-al-2026-controlled-by-female-hormones-a-qualitative-interview-study-of-swedish-women-s-experiences-of.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/mctaggart-et-al-2026-controlled-by-female-hormones-a-qualitative-interview-study-of-swedish-women-s-experiences-of.pdf</t>
         </is>
       </c>
       <c r="D99" t="inlineStr" s="0">
@@ -7468,7 +7468,7 @@
       </c>
       <c r="C100" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/nagata_2026_oi_260668_1783701523.89945.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/nagata_2026_oi_260668_1783701523.89945.pdf</t>
         </is>
       </c>
       <c r="D100" t="inlineStr" s="0">
@@ -7505,7 +7505,7 @@
       </c>
       <c r="C101" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/nutrients-18-01625.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/nutrients-18-01625.pdf</t>
         </is>
       </c>
       <c r="D101" t="inlineStr" s="0">
@@ -7542,7 +7542,7 @@
       </c>
       <c r="C102" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/nutrients-18-02357.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/nutrients-18-02357.pdf</t>
         </is>
       </c>
       <c r="D102" t="inlineStr" s="0">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="C103" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/nutrients-18-02664-v2.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/nutrients-18-02664-v2.pdf</t>
         </is>
       </c>
       <c r="D103" t="inlineStr" s="0">
@@ -7616,7 +7616,7 @@
       </c>
       <c r="C104" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/pardo-palenzuela-et-al-2025-cognitive-profile-of-adhd-in-older-adults-a-systematic-review.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/pardo-palenzuela-et-al-2025-cognitive-profile-of-adhd-in-older-adults-a-systematic-review.pdf</t>
         </is>
       </c>
       <c r="D104" t="inlineStr" s="0">
@@ -7653,7 +7653,7 @@
       </c>
       <c r="C105" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/pathan-et-al-2026-impact-of-medication-therapy-on-social-behavioral-and-employment-outcomes-in-adults-with-adhd.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/pathan-et-al-2026-impact-of-medication-therapy-on-social-behavioral-and-employment-outcomes-in-adults-with-adhd.pdf</t>
         </is>
       </c>
       <c r="D105" t="inlineStr" s="0">
@@ -7690,7 +7690,7 @@
       </c>
       <c r="C106" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/peerj-20603.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/peerj-20603.pdf</t>
         </is>
       </c>
       <c r="D106" t="inlineStr" s="0">
@@ -7727,7 +7727,7 @@
       </c>
       <c r="C107" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/pierotti-jayakody-2025-maternal-attention-deficit-hyperactivity-disorder-and-perinatal-depression-a-systematic-review.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/pierotti-jayakody-2025-maternal-attention-deficit-hyperactivity-disorder-and-perinatal-depression-a-systematic-review.pdf</t>
         </is>
       </c>
       <c r="D107" t="inlineStr" s="0">
@@ -7764,7 +7764,7 @@
       </c>
       <c r="C108" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/quality-assessment-of-adhd-related-short-videos-on-chinese.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/quality-assessment-of-adhd-related-short-videos-on-chinese.pdf</t>
         </is>
       </c>
       <c r="D108" t="inlineStr" s="0">
@@ -7801,7 +7801,7 @@
       </c>
       <c r="C109" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/rafael-et-al-2026-attention-deficit-hyperactivity-disorder-(adhd)-related-strengths-in-adults-a-scoping-review.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/rafael-et-al-2026-attention-deficit-hyperactivity-disorder-(adhd)-related-strengths-in-adults-a-scoping-review.pdf</t>
         </is>
       </c>
       <c r="D109" t="inlineStr" s="0">
@@ -7838,7 +7838,7 @@
       </c>
       <c r="C110" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/resprot-2026-1-e79150.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/resprot-2026-1-e79150.pdf</t>
         </is>
       </c>
       <c r="D110" t="inlineStr" s="0">
@@ -7875,7 +7875,7 @@
       </c>
       <c r="C111" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00406-025-02148-z.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00406-025-02148-z.pdf</t>
         </is>
       </c>
       <c r="D111" t="inlineStr" s="0">
@@ -7912,7 +7912,7 @@
       </c>
       <c r="C112" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00406-025-02162-1.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00406-025-02162-1.pdf</t>
         </is>
       </c>
       <c r="D112" t="inlineStr" s="0">
@@ -7949,7 +7949,7 @@
       </c>
       <c r="C113" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00787-025-02822-6.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00787-025-02822-6.pdf</t>
         </is>
       </c>
       <c r="D113" t="inlineStr" s="0">
@@ -7986,7 +7986,7 @@
       </c>
       <c r="C114" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00787-025-02842-2.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00787-025-02842-2.pdf</t>
         </is>
       </c>
       <c r="D114" t="inlineStr" s="0">
@@ -8023,7 +8023,7 @@
       </c>
       <c r="C115" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00787-025-02904-5.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00787-025-02904-5.pdf</t>
         </is>
       </c>
       <c r="D115" t="inlineStr" s="0">
@@ -8060,7 +8060,7 @@
       </c>
       <c r="C116" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00787-025-02906-3.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00787-025-02906-3.pdf</t>
         </is>
       </c>
       <c r="D116" t="inlineStr" s="0">
@@ -8097,7 +8097,7 @@
       </c>
       <c r="C117" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00787-025-02947-8.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00787-025-02947-8.pdf</t>
         </is>
       </c>
       <c r="D117" t="inlineStr" s="0">
@@ -8134,7 +8134,7 @@
       </c>
       <c r="C118" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00787-026-02987-8.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00787-026-02987-8.pdf</t>
         </is>
       </c>
       <c r="D118" t="inlineStr" s="0">
@@ -8171,7 +8171,7 @@
       </c>
       <c r="C119" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s00787-026-03059-7.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s00787-026-03059-7.pdf</t>
         </is>
       </c>
       <c r="D119" t="inlineStr" s="0">
@@ -8208,7 +8208,7 @@
       </c>
       <c r="C120" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s10508-026-03448-8.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s10508-026-03448-8.pdf</t>
         </is>
       </c>
       <c r="D120" t="inlineStr" s="0">
@@ -8245,7 +8245,7 @@
       </c>
       <c r="C121" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s10567-026-00563-9.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s10567-026-00563-9.pdf</t>
         </is>
       </c>
       <c r="D121" t="inlineStr" s="0">
@@ -8282,7 +8282,7 @@
       </c>
       <c r="C122" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s10578-024-01732-z.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s10578-024-01732-z.pdf</t>
         </is>
       </c>
       <c r="D122" t="inlineStr" s="0">
@@ -8319,7 +8319,7 @@
       </c>
       <c r="C123" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s10802-026-01488-1.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s10802-026-01488-1.pdf</t>
         </is>
       </c>
       <c r="D123" t="inlineStr" s="0">
@@ -8356,7 +8356,7 @@
       </c>
       <c r="C124" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s10803-024-06410-6.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s10803-024-06410-6.pdf</t>
         </is>
       </c>
       <c r="D124" t="inlineStr" s="0">
@@ -8393,7 +8393,7 @@
       </c>
       <c r="C125" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s10803-024-06623-9.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s10803-024-06623-9.pdf</t>
         </is>
       </c>
       <c r="D125" t="inlineStr" s="0">
@@ -8430,7 +8430,7 @@
       </c>
       <c r="C126" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s10803-024-06682-y.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s10803-024-06682-y.pdf</t>
         </is>
       </c>
       <c r="D126" t="inlineStr" s="0">
@@ -8467,7 +8467,7 @@
       </c>
       <c r="C127" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s11096-026-02184-2.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s11096-026-02184-2.pdf</t>
         </is>
       </c>
       <c r="D127" t="inlineStr" s="0">
@@ -8504,7 +8504,7 @@
       </c>
       <c r="C128" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s11126-025-10185-z.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s11126-025-10185-z.pdf</t>
         </is>
       </c>
       <c r="D128" t="inlineStr" s="0">
@@ -8541,7 +8541,7 @@
       </c>
       <c r="C129" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s11136-026-04244-6.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s11136-026-04244-6.pdf</t>
         </is>
       </c>
       <c r="D129" t="inlineStr" s="0">
@@ -8578,7 +8578,7 @@
       </c>
       <c r="C130" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12325-026-03638-9.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12325-026-03638-9.pdf</t>
         </is>
       </c>
       <c r="D130" t="inlineStr" s="0">
@@ -8615,7 +8615,7 @@
       </c>
       <c r="C131" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12887-025-06465-z.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12887-025-06465-z.pdf</t>
         </is>
       </c>
       <c r="D131" t="inlineStr" s="0">
@@ -8652,7 +8652,7 @@
       </c>
       <c r="C132" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12887-026-06646-4.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12887-026-06646-4.pdf</t>
         </is>
       </c>
       <c r="D132" t="inlineStr" s="0">
@@ -8689,7 +8689,7 @@
       </c>
       <c r="C133" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12887-026-06963-8.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12887-026-06963-8.pdf</t>
         </is>
       </c>
       <c r="D133" t="inlineStr" s="0">
@@ -8726,7 +8726,7 @@
       </c>
       <c r="C134" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12888-026-07953-x.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12888-026-07953-x.pdf</t>
         </is>
       </c>
       <c r="D134" t="inlineStr" s="0">
@@ -8763,7 +8763,7 @@
       </c>
       <c r="C135" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12888-026-08293-6.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12888-026-08293-6.pdf</t>
         </is>
       </c>
       <c r="D135" t="inlineStr" s="0">
@@ -8800,7 +8800,7 @@
       </c>
       <c r="C136" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12888-026-08296-3.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12888-026-08296-3.pdf</t>
         </is>
       </c>
       <c r="D136" t="inlineStr" s="0">
@@ -8837,7 +8837,7 @@
       </c>
       <c r="C137" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12889-026-27631-7.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12889-026-27631-7.pdf</t>
         </is>
       </c>
       <c r="D137" t="inlineStr" s="0">
@@ -8874,7 +8874,7 @@
       </c>
       <c r="C138" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s12903-026-07704-0.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s12903-026-07704-0.pdf</t>
         </is>
       </c>
       <c r="D138" t="inlineStr" s="0">
@@ -8911,7 +8911,7 @@
       </c>
       <c r="C139" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s40001-025-03711-z.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s40001-025-03711-z.pdf</t>
         </is>
       </c>
       <c r="D139" t="inlineStr" s="0">
@@ -8948,7 +8948,7 @@
       </c>
       <c r="C140" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s40359-026-04637-9.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s40359-026-04637-9.pdf</t>
         </is>
       </c>
       <c r="D140" t="inlineStr" s="0">
@@ -8985,7 +8985,7 @@
       </c>
       <c r="C141" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s40359-026-05200-2.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s40359-026-05200-2.pdf</t>
         </is>
       </c>
       <c r="D141" t="inlineStr" s="0">
@@ -9022,7 +9022,7 @@
       </c>
       <c r="C142" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41380-025-03178-8.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41380-025-03178-8.pdf</t>
         </is>
       </c>
       <c r="D142" t="inlineStr" s="0">
@@ -9059,7 +9059,7 @@
       </c>
       <c r="C143" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41380-025-03242-3.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41380-025-03242-3.pdf</t>
         </is>
       </c>
       <c r="D143" t="inlineStr" s="0">
@@ -9096,7 +9096,7 @@
       </c>
       <c r="C144" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41380-026-03645-w.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41380-026-03645-w.pdf</t>
         </is>
       </c>
       <c r="D144" t="inlineStr" s="0">
@@ -9133,7 +9133,7 @@
       </c>
       <c r="C145" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41390-025-04325-1.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41390-025-04325-1.pdf</t>
         </is>
       </c>
       <c r="D145" t="inlineStr" s="0">
@@ -9170,7 +9170,7 @@
       </c>
       <c r="C146" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41398-026-03972-0.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41398-026-03972-0.pdf</t>
         </is>
       </c>
       <c r="D146" t="inlineStr" s="0">
@@ -9207,7 +9207,7 @@
       </c>
       <c r="C147" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41398-026-04151-x.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41398-026-04151-x.pdf</t>
         </is>
       </c>
       <c r="D147" t="inlineStr" s="0">
@@ -9244,7 +9244,7 @@
       </c>
       <c r="C148" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41398-026-04166-4.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41398-026-04166-4.pdf</t>
         </is>
       </c>
       <c r="D148" t="inlineStr" s="0">
@@ -9281,7 +9281,7 @@
       </c>
       <c r="C149" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41598-025-34570-7.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41598-025-34570-7.pdf</t>
         </is>
       </c>
       <c r="D149" t="inlineStr" s="0">
@@ -9318,7 +9318,7 @@
       </c>
       <c r="C150" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41598-026-41493-4.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41598-026-41493-4.pdf</t>
         </is>
       </c>
       <c r="D150" t="inlineStr" s="0">
@@ -9355,7 +9355,7 @@
       </c>
       <c r="C151" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/s41598-026-54609-7.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/s41598-026-54609-7.pdf</t>
         </is>
       </c>
       <c r="D151" t="inlineStr" s="0">
@@ -9392,7 +9392,7 @@
       </c>
       <c r="C152" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/sensors-26-05684.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/sensors-26-05684.pdf</t>
         </is>
       </c>
       <c r="D152" t="inlineStr" s="0">
@@ -9429,7 +9429,7 @@
       </c>
       <c r="C153" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/spencer-et-al-2025-equity-centered-development-of-a-community-health-worker-intervention-to-improve-engagement-in-care.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/spencer-et-al-2025-equity-centered-development-of-a-community-health-worker-intervention-to-improve-engagement-in-care.pdf</t>
         </is>
       </c>
       <c r="D153" t="inlineStr" s="0">
@@ -9466,7 +9466,7 @@
       </c>
       <c r="C154" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/taylor-et-al-2026-parent-perspectives-on-barriers-to-behavioral-health-services-for-children-with-adhd.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/taylor-et-al-2026-parent-perspectives-on-barriers-to-behavioral-health-services-for-children-with-adhd.pdf</t>
         </is>
       </c>
       <c r="D154" t="inlineStr" s="0">
@@ -9503,7 +9503,7 @@
       </c>
       <c r="C155" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/the-association-between-asthma-and-adhd-in-children-and.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/the-association-between-asthma-and-adhd-in-children-and.pdf</t>
         </is>
       </c>
       <c r="D155" t="inlineStr" s="0">
@@ -9540,7 +9540,7 @@
       </c>
       <c r="C156" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/the-relationship-between-problematic-social-media-use-and.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/the-relationship-between-problematic-social-media-use-and.pdf</t>
         </is>
       </c>
       <c r="D156" t="inlineStr" s="0">
@@ -9577,7 +9577,7 @@
       </c>
       <c r="C157" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/what-predicts-attention-deficithyperactivity-disorder.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/what-predicts-attention-deficithyperactivity-disorder.pdf</t>
         </is>
       </c>
       <c r="D157" t="inlineStr" s="0">
@@ -9614,7 +9614,7 @@
       </c>
       <c r="C158" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/zhang-et-al-2025-effects-of-exercise-on-hyperactivity-impulsivity-and-inhibitory-control-at-behavioral-and.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/zhang-et-al-2025-effects-of-exercise-on-hyperactivity-impulsivity-and-inhibitory-control-at-behavioral-and.pdf</t>
         </is>
       </c>
       <c r="D158" t="inlineStr" s="0">
@@ -9651,7 +9651,7 @@
       </c>
       <c r="C159" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/zhang-et-al-2026-optimizing-exercise-interventions-for-motor-skills-enhancement-in-attention-deficit-hyperactivity.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/zhang-et-al-2026-optimizing-exercise-interventions-for-motor-skills-enhancement-in-attention-deficit-hyperactivity.pdf</t>
         </is>
       </c>
       <c r="D159" t="inlineStr" s="0">
@@ -9688,7 +9688,7 @@
       </c>
       <c r="C160" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">full_texts/öztürk-et-al-2026-increased-serum-netrin-1-levels-among-children-diagnosed-with-adhd.pdf</t>
+          <t xml:space="preserve">../2026 ADHD Papers/öztürk-et-al-2026-increased-serum-netrin-1-levels-among-children-diagnosed-with-adhd.pdf</t>
         </is>
       </c>
       <c r="D160" t="inlineStr" s="0">
@@ -9840,7 +9840,7 @@
       </c>
       <c r="B10" t="inlineStr" s="0">
         <is>
-          <t xml:space="preserve">Graph SHA-256, every supplied PDF SHA-256, text hashes and reviewed corpus hash are checked. New/changed graphs or source PDFs require reassessment before rebuilding. full_texts is a relative directory link to the original supplied corpus; keep these folders beside 2026 ADHD Papers.</t>
+          <t xml:space="preserve">Graph SHA-256, every supplied PDF SHA-256, text hashes and reviewed corpus hash are checked. New/changed graphs or source PDFs require reassessment before rebuilding. PDF references point directly to the committed 2026 ADHD Papers folder through relative paths; no directory links are required. Git checkout newline conversions are accepted for reviewed text files only.</t>
         </is>
       </c>
     </row>

</xml_diff>